<commit_message>
update param names in source files
</commit_message>
<xml_diff>
--- a/sources/macro/gdp/US Bureau of Economic Analysis GDP deflator.xlsx
+++ b/sources/macro/gdp/US Bureau of Economic Analysis GDP deflator.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\CIMS\dev\cims-models\sources\macro\gdp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E768ED6-90F7-4A41-9B58-09B01618BCBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD344441-6FD9-4E53-8885-2E1871A430CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34935" yWindow="3045" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029" iterate="1" calcOnSave="0"/>
+  <calcPr calcId="191029" calcOnSave="0"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -697,13 +697,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AH33"/>
-  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:34" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -741,7 +742,7 @@
       <c r="AG1" s="3"/>
       <c r="AH1" s="3"/>
     </row>
-    <row r="2" spans="1:34" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -779,7 +780,7 @@
       <c r="AG2" s="3"/>
       <c r="AH2" s="3"/>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
@@ -817,7 +818,7 @@
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -855,7 +856,7 @@
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>4</v>
       </c>
@@ -957,12 +958,12 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>37</v>
       </c>
@@ -1066,7 +1067,7 @@
         <v>118.49</v>
       </c>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>39</v>
       </c>
@@ -1170,7 +1171,7 @@
         <v>115.53</v>
       </c>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>41</v>
       </c>
@@ -1274,7 +1275,7 @@
         <v>98.89</v>
       </c>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>43</v>
       </c>
@@ -1378,7 +1379,7 @@
         <v>91.186999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>45</v>
       </c>
@@ -1482,7 +1483,7 @@
         <v>102.839</v>
       </c>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>47</v>
       </c>
@@ -1586,7 +1587,7 @@
         <v>124.215</v>
       </c>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>49</v>
       </c>
@@ -1690,7 +1691,7 @@
         <v>113.825</v>
       </c>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>51</v>
       </c>
@@ -1794,7 +1795,7 @@
         <v>115.387</v>
       </c>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>53</v>
       </c>
@@ -1898,7 +1899,7 @@
         <v>106.44</v>
       </c>
     </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>55</v>
       </c>
@@ -2002,7 +2003,7 @@
         <v>127.67400000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>57</v>
       </c>
@@ -2106,7 +2107,7 @@
         <v>97.686999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>59</v>
       </c>
@@ -2210,7 +2211,7 @@
         <v>105.595</v>
       </c>
     </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>61</v>
       </c>
@@ -2314,7 +2315,7 @@
         <v>153.74799999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>63</v>
       </c>
@@ -2418,7 +2419,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>66</v>
       </c>
@@ -2522,7 +2523,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -2626,7 +2627,7 @@
         <v>107.54900000000001</v>
       </c>
     </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>70</v>
       </c>
@@ -2730,7 +2731,7 @@
         <v>100.913</v>
       </c>
     </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>72</v>
       </c>
@@ -2834,7 +2835,7 @@
         <v>121.42</v>
       </c>
     </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -2938,7 +2939,7 @@
         <v>94.613</v>
       </c>
     </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>76</v>
       </c>
@@ -3042,7 +3043,7 @@
         <v>90.536000000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>77</v>
       </c>
@@ -3146,7 +3147,7 @@
         <v>115.53400000000001</v>
       </c>
     </row>
-    <row r="29" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>78</v>
       </c>
@@ -3250,7 +3251,7 @@
         <v>120.039</v>
       </c>
     </row>
-    <row r="30" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>80</v>
       </c>
@@ -3354,7 +3355,7 @@
         <v>116.04900000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>82</v>
       </c>
@@ -3458,7 +3459,7 @@
         <v>114.104</v>
       </c>
     </row>
-    <row r="32" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>84</v>
       </c>
@@ -3562,7 +3563,7 @@
         <v>119.10599999999999</v>
       </c>
     </row>
-    <row r="33" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>86</v>
       </c>

</xml_diff>